<commit_message>
publish: sync from 正本 2026-09-24T22:29:11Z
</commit_message>
<xml_diff>
--- a/plugins/osi-finance/assets/templates/請求管理台帳_テンプレート.xlsx
+++ b/plugins/osi-finance/assets/templates/請求管理台帳_テンプレート.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方_請求管理台帳" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="発行者設定" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="契約マスタ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月次請求スケジュール" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="雛形マスタ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月次請求スケジュール" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,15 +31,13 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -47,16 +46,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -64,36 +58,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,52 +437,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="140" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>請求管理台帳テンプレート（AR・もらう側）  ※OSI Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>請求管理台帳 テンプレート（AR・もらう側）  ※OSI Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>・ファイル名は『請求管理台帳.xlsx』（または settings の LEDGER_BILLING_FILE）にして置きます。</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>・このファイルを自組織の Drive `31.請求管理/02.送付請求書/` に『請求管理台帳.xlsx』として配置します。</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>・置き場所：経理フォルダ（osi-profile.md の paths.finance ＝ 拡張の設定「台帳フォルダ」xlsx_ledger_dir）。共通マスタ・請求管理台帳・支払管理台帳・仕訳台帳・コンソールを開く.html を同じフォルダに置く。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>・黄色＝記入例。実データを入れる前に削除してください。</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>・データ行は空です。記入例は下にだけ書いてあります（台帳の行に例を置くと、月初の請求処理などが本物として拾います）。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>・発行者設定は keiri-settings の値と一致させます（請求書PDFに反映）。</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>・列はヘッダー名で読みます。列の追加・並べ替えはかまいませんが、列名は変えないでください。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>・契約マスタ＝1契約1行（契約ID=C-連番）。月次請求スケジュール＝対象月ごとの請求予定。</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>・分からない値は空欄にして、理由を備考に書きます（「要確認」などの文字で埋めない）。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>・採番 INV-YYYY-MM-連番3桁は keiri-invoice 発行時に確定。</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>・仕様の正本：プラグインの assets/schema/data-layout.yaml。テンプレートは assets/scripts/build_templates.py で生成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>・発行者設定：値は osi-finance-setup が osi-finance-settings.md から埋めます（assets/scripts/fill_issuer_settings.py）。空欄のままでは請求書を発行しません（osi-finance-invoice が止めて知らせます）。settings を変えたら埋め直します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>・契約マスタ：1契約1行。契約ID=AR-C-001（受注）／AP-C-001（発注）。会社の名前・住所・宛先は持たず、取引先ID で共通マスタの取引先マスタを引きます。状態=締結済 の行だけが請求予定に展開されます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>・雛形マスタ：契約書の雛形（TPL-001…）。osi-finance-contract-draft が登録します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>・月次請求スケジュール：1行=1請求。osi-finance-contract-intake が契約から展開し、請求書番号（INV-YYYY-MM-連番3桁、YYYY-MM=請求月）は osi-finance-invoice が発行するときに振ります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>・前受・消化型（回数券など）を使う組織だけ「消化記録」タブを足します（settings §4-4）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>記入例（参考。台帳には書かない）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  契約マスタ：契約ID=AR-C-001 / 取引先=サンプル / 契約種別=業務委託(準委任) / 金額区分=月額固定 / 月額(税込)=220000 / 税率=10% / 契約開始=2026-04-01 / 契約終了=2027-03-31 / 取引先ID=P-001 / 方向=受注 / 状態=締結済 / 出所=手動</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  月次請求スケジュール：契約ID=AR-C-001 / 対象月=2026-04 / 件名=業務委託（2026年4月分） / 請求額(税込)=220000 / 請求ステータス=未請求</t>
         </is>
       </c>
     </row>
@@ -519,26 +562,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>値</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
@@ -550,14 +593,9 @@
           <t>発行者名義</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>（自社名を入力）</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>keiri-settings と一致</t>
+          <t>settings の ISSUER_NAME から setup が記入</t>
         </is>
       </c>
     </row>
@@ -567,9 +605,9 @@
           <t>登録番号</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>（適格請求書 登録番号 T+13桁）</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>T＋13桁。settings の ISSUER_INVOICE_REG_NO から setup が記入</t>
         </is>
       </c>
     </row>
@@ -579,9 +617,9 @@
           <t>郵便番号</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>（例 000-0000）</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>settings の ISSUER_POSTAL_CODE から setup が記入</t>
         </is>
       </c>
     </row>
@@ -591,9 +629,9 @@
           <t>住所</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>（本店所在地）</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>settings の ISSUER_ADDRESS から setup が記入</t>
         </is>
       </c>
     </row>
@@ -603,9 +641,9 @@
           <t>振込先 銀行</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>（銀行名）</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>settings の BANK_NAME から setup が記入</t>
         </is>
       </c>
     </row>
@@ -615,9 +653,9 @@
           <t>振込先 支店</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>（支店名・店番）</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>settings の BANK_BRANCH から setup が記入</t>
         </is>
       </c>
     </row>
@@ -627,9 +665,9 @@
           <t>預金種別</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>普通</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>settings の ACCOUNT_TYPE から setup が記入</t>
         </is>
       </c>
     </row>
@@ -639,9 +677,9 @@
           <t>口座番号</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>（口座番号）</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>settings の ACCOUNT_NUMBER から setup が記入</t>
         </is>
       </c>
     </row>
@@ -651,72 +689,135 @@
           <t>口座名義</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>（口座名義）</t>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>settings の ACCOUNT_HOLDER から setup が記入</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>消費税率</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>10%</t>
+          <t>振込手数料</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>標準税率</t>
+          <t>settings の TRANSFER_FEE_BEARER から setup が記入</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>採番ルール</t>
+          <t>消費税率</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>INV-YYYY-MM-連番3桁</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>対象月＋月内連番</t>
+          <t>settings の CONSUMPTION_TAX_RATE から setup が記入</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>支払サイト</t>
+          <t>採番ルール</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>月末締め翌月末払い</t>
+          <t>INV-YYYY-MM-連番3桁</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>請求日=対象月翌月1日/支払期限=翌月末</t>
+          <t>settings の AR_NUMBERING から setup が記入</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>振込手数料</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>お客様負担</t>
+          <t>支払サイト</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>settings の AR_PAYMENT_TERMS から setup が記入</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>電子署名</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>settings の ESIGN から setup が記入</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>会計SaaS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>settings の ACCOUNTING_SYNC から setup が記入</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>銀行明細突合</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>settings の BANK_RECON から setup が記入</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>金額区分</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>月額固定=monthly; 一括=lump; 都度=variable</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>settings の BILLING_PATTERNS から setup が記入</t>
         </is>
       </c>
     </row>
@@ -731,30 +832,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="4" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="28" customWidth="1" min="19" max="19"/>
-    <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" style="4" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" style="4" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" style="4" min="22" max="22"/>
+    <col width="26" customWidth="1" style="4" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -770,194 +877,142 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>正式名称</t>
+          <t>契約種別</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>郵便番号</t>
+          <t>契約内容</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>住所</t>
+          <t>金額区分</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>請求先To</t>
+          <t>月額(税込)</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Toアドレス</t>
+          <t>一括額(税込)</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>数量</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>CCアドレス</t>
+          <t>単価(税込)</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>契約種別</t>
+          <t>有効期限</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>契約内容</t>
+          <t>税率</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>金額区分</t>
+          <t>契約開始</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
-          <t>月額(税込)</t>
+          <t>契約終了</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>一括額(税込)</t>
+          <t>支払サイト</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
         <is>
-          <t>税率</t>
+          <t>契約書ファイル</t>
         </is>
       </c>
       <c r="P1" s="3" t="inlineStr">
         <is>
-          <t>契約開始</t>
+          <t>旧ID</t>
         </is>
       </c>
       <c r="Q1" s="3" t="inlineStr">
         <is>
-          <t>契約終了</t>
+          <t>備考</t>
         </is>
       </c>
       <c r="R1" s="3" t="inlineStr">
         <is>
-          <t>支払サイト</t>
+          <t>取引先ID</t>
         </is>
       </c>
       <c r="S1" s="3" t="inlineStr">
         <is>
-          <t>契約書ファイル</t>
+          <t>方向</t>
         </is>
       </c>
       <c r="T1" s="3" t="inlineStr">
         <is>
-          <t>ステータス</t>
+          <t>状態</t>
         </is>
       </c>
       <c r="U1" s="3" t="inlineStr">
         <is>
-          <t>備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>C-001</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>（記入例）サンプル商事</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>株式会社サンプル商事</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>000-0000</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>東京都…</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>担当者名</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>aaa@example.com</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>業務委託(準委任)</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>CAIO業務</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>月額固定</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>220000</v>
-      </c>
-      <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="inlineStr">
-        <is>
-          <t>月末締め翌月末払い</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="inlineStr">
-        <is>
-          <t>00.契約書/サンプル商事_業務委託_20260401.pdf</t>
-        </is>
-      </c>
-      <c r="T2" s="4" t="inlineStr">
-        <is>
-          <t>有効</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>記入例。実運用前に削除</t>
+          <t>出所</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>雛形ID</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>envelope_id</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>作成者</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>作成日時</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>更新者</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>更新日時</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="S2:S2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"受注,発注"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"ドラフト,送付済,締結済"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"手動,Gmail取込,実績から"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -968,27 +1023,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="4" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>雛形ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>雛形名</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>用途メモ</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>ファイルパス</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>登録日</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>登録元</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>使用回数</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>登録者</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>更新者</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>更新日時</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"受注用,発注用,共通"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"AI生成,実契約からの雛形化"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="4" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" style="4" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" style="4" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" style="4" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
           <t>契約ID</t>
         </is>
       </c>
@@ -1049,69 +1203,51 @@
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
+          <t>旧ID</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
           <t>備考</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>送付日</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>C-001</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>（記入例）サンプル商事</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>CAIO業務（2026年4月分）</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>220000</v>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>INV-2026-05-001</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>未請求</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>記入例。実運用前に削除</t>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>突合結果</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>突合日時</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>作成者</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>作成日時</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>更新者</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>更新日時</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="仕様外の値" error="data-layout.yaml の values 以外の値です" type="list" errorStyle="warning">
+      <formula1>"未請求,下書き済,請求済,入金済,対象外,要確認(過去・番号なし)"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>